<commit_message>
v1.1: operacion potencia con ciclo for (solicitud de cambio CR-001)
- Nuevo metodo potencia(a, b) con for, valida exponente negativo y desbordamiento
- Pruebas QA022-QA027 y regresion de QA001-QA021 registradas en PruebasUnitarias.xlsx
</commit_message>
<xml_diff>
--- a/PruebasUnitarias.xlsx
+++ b/PruebasUnitarias.xlsx
@@ -1625,82 +1625,326 @@
       </c>
     </row>
     <row r="24" ht="189.55" customHeight="1" s="12">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="17" t="n"/>
-      <c r="K24" s="16" t="n"/>
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>QA022</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Potencia con exponente positivo (ciclo for)</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>2 y 10</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="n">
+        <v>1024</v>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>2 ^ 10 = 1024</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="162.65" customHeight="1" s="12">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="17" t="n"/>
-      <c r="K25" s="16" t="n"/>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>QA023</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Potencia con exponente cero</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>5 y 0</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>5 ^ 0 = 1</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J25" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="68.65000000000001" customHeight="1" s="12">
-      <c r="A26" s="15" t="n"/>
-      <c r="B26" s="15" t="n"/>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="17" t="n"/>
-      <c r="K26" s="16" t="n"/>
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>QA024</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Potencia con base negativa y exponente impar</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>-2 y 3</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>-8</v>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>-2 ^ 3 = -8</t>
+        </is>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="135.8" customHeight="1" s="12">
-      <c r="A27" s="15" t="n"/>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
-      <c r="I27" s="15" t="n"/>
-      <c r="J27" s="17" t="n"/>
-      <c r="K27" s="16" t="n"/>
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>QA025</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Potencia con base cero</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>0 y 4</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>0 ^ 4 = 0</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="95.5" customHeight="1" s="12">
-      <c r="A28" s="15" t="n"/>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
-      <c r="I28" s="15" t="n"/>
-      <c r="J28" s="17" t="n"/>
-      <c r="K28" s="16" t="n"/>
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>QA026</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Potencia con exponente negativo</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>2 y -1</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Potencia: operacion no valida, el exponente no puede ser negativo.</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Potencia: operacion no valida, el exponente no puede ser negativo.</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="82.05" customHeight="1" s="12">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
-      <c r="I29" s="15" t="n"/>
-      <c r="J29" s="17" t="n"/>
-      <c r="K29" s="16" t="n"/>
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>QA027</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Unitario</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>Juan Camilo Lopez</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Potencia que supera el rango de long (desbordamiento)</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>Clase OperacionesAritmeticas, metodo potencia</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>10 y 19</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>Potencia: operacion no valida, el resultado supera el rango de un entero.</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Potencia: operacion no valida, el resultado supera el rango de un entero.</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno, prueba aprobada</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="12">
       <c r="A31" s="18" t="inlineStr">
@@ -1756,7 +2000,7 @@
     <row r="36" ht="19.5" customHeight="1" s="12">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>Nota: tests unitarios ejecutados manualmente por consola (java OperacionesAritmeticas), un caso por ejecucion, verificando la linea del metodo probado.</t>
+          <t>Nota: tests unitarios ejecutados manualmente por consola (java OperacionesAritmeticas), un caso por ejecucion, verificando la linea del metodo probado. QA022 a QA027 corresponden a la solicitud de cambio CR-001 (potencia, v1.1).</t>
         </is>
       </c>
     </row>

</xml_diff>